<commit_message>
extent report config changes
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/simple.xlsx
+++ b/src/test/resources/testData/simple.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07EA50E2-FD17-4252-B051-99410B85D4BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77DE3283-BDEB-4241-834D-5B03EE8458B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="631" uniqueCount="120">
   <si>
     <t>Runmode</t>
   </si>
@@ -366,7 +366,22 @@
     <t>admin123</t>
   </si>
   <si>
-    <t>loginToHrm</t>
+    <t>Module</t>
+  </si>
+  <si>
+    <t>Performance</t>
+  </si>
+  <si>
+    <t>username</t>
+  </si>
+  <si>
+    <t>loginToPerformanceModule</t>
+  </si>
+  <si>
+    <t>loginToTimeModule</t>
+  </si>
+  <si>
+    <t>Time</t>
   </si>
 </sst>
 </file>
@@ -2816,7 +2831,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6867381B-BC0D-48B4-97F8-7942607A6379}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.77734375" customWidth="1"/>
@@ -2828,7 +2843,7 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2843,13 +2858,13 @@
         <v>14</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>23</v>
+        <v>116</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>25</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -2865,8 +2880,51 @@
       <c r="D3" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="E3" t="s">
-        <v>110</v>
+      <c r="E3" s="4" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>119</v>
       </c>
     </row>
   </sheetData>
@@ -2874,6 +2932,9 @@
     <hyperlink ref="B3" r:id="rId1" xr:uid="{C877C554-C839-453A-827C-8C58F42EC787}"/>
     <hyperlink ref="C3" r:id="rId2" display="prabhudatta.c@tadigital.com" xr:uid="{30200C7E-5999-4DF2-8038-487829621B70}"/>
     <hyperlink ref="D3" r:id="rId3" display="Welcome@1234" xr:uid="{07219809-3D3C-4110-AB6F-58416FAEFE83}"/>
+    <hyperlink ref="B7" r:id="rId4" xr:uid="{96D51270-707E-46C0-A767-2C625E170FC7}"/>
+    <hyperlink ref="C7" r:id="rId5" display="prabhudatta.c@tadigital.com" xr:uid="{A2028C79-5340-4FD5-8652-D0A5526B04F4}"/>
+    <hyperlink ref="D7" r:id="rId6" display="Welcome@1234" xr:uid="{07B4274B-608A-4BBF-AA43-8664B98A04F9}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>